<commit_message>
fix: update HPE bid line item output
</commit_message>
<xml_diff>
--- a/samples/outputs/HPE_Deal_9500000001_v2_NoCalculation.xlsx
+++ b/samples/outputs/HPE_Deal_9500000001_v2_NoCalculation.xlsx
@@ -114,9 +114,6 @@
     <x:t>MSL 2024 2xTLO-9 SAS</x:t>
   </x:si>
   <x:si>
-    <x:t>Max Qty: 1</x:t>
-  </x:si>
-  <x:si>
     <x:t>1.01</x:t>
   </x:si>
   <x:si>
@@ -183,12 +180,18 @@
     <x:t>1.08</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4B2A3#QC1</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE MSL TapeAssure Adv Lic Support</x:t>
   </x:si>
   <x:si>
     <x:t>1.09</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4B2A3#80N</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE MSL2024 Library Support</x:t>
   </x:si>
   <x:si>
@@ -222,6 +225,9 @@
     <x:t>2.03</x:t>
   </x:si>
   <x:si>
+    <x:t>R7M24A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Factory Integrated</x:t>
   </x:si>
   <x:si>
@@ -237,6 +243,9 @@
     <x:t>2.05</x:t>
   </x:si>
   <x:si>
+    <x:t>BB983A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>FACTORY INTEGRATED</x:t>
   </x:si>
   <x:si>
@@ -261,6 +270,9 @@
     <x:t>2.08</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4A6A3#YHL</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE StoreOnce 3660 80TB Base System Supp</x:t>
   </x:si>
   <x:si>
@@ -276,6 +288,9 @@
     <x:t>2.10</x:t>
   </x:si>
   <x:si>
+    <x:t>HA124A1#5VF</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE StoreOnce 36xx Stup SVC</x:t>
   </x:si>
   <x:si>
@@ -309,6 +324,9 @@
     <x:t>3.02</x:t>
   </x:si>
   <x:si>
+    <x:t>P52499-B21#UUF</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.03</x:t>
   </x:si>
   <x:si>
@@ -321,6 +339,9 @@
     <x:t>3.04</x:t>
   </x:si>
   <x:si>
+    <x:t>P67079-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Factory integrated</x:t>
   </x:si>
   <x:si>
@@ -336,6 +357,9 @@
     <x:t>3.06</x:t>
   </x:si>
   <x:si>
+    <x:t>P64706-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.07</x:t>
   </x:si>
   <x:si>
@@ -348,6 +372,9 @@
     <x:t>3.08</x:t>
   </x:si>
   <x:si>
+    <x:t>P48895-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.09</x:t>
   </x:si>
   <x:si>
@@ -360,6 +387,9 @@
     <x:t>3.10</x:t>
   </x:si>
   <x:si>
+    <x:t>804398-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.11</x:t>
   </x:si>
   <x:si>
@@ -372,6 +402,9 @@
     <x:t>3.12</x:t>
   </x:si>
   <x:si>
+    <x:t>P26259-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.13</x:t>
   </x:si>
   <x:si>
@@ -384,6 +417,9 @@
     <x:t>3.14</x:t>
   </x:si>
   <x:si>
+    <x:t>P01366-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.15</x:t>
   </x:si>
   <x:si>
@@ -396,6 +432,9 @@
     <x:t>3.16</x:t>
   </x:si>
   <x:si>
+    <x:t>P48918-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.17</x:t>
   </x:si>
   <x:si>
@@ -408,6 +447,9 @@
     <x:t>3.18</x:t>
   </x:si>
   <x:si>
+    <x:t>P58335-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.19</x:t>
   </x:si>
   <x:si>
@@ -420,6 +462,9 @@
     <x:t>3.20</x:t>
   </x:si>
   <x:si>
+    <x:t>P51181-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.21</x:t>
   </x:si>
   <x:si>
@@ -432,6 +477,9 @@
     <x:t>3.22</x:t>
   </x:si>
   <x:si>
+    <x:t>P48908-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.23</x:t>
   </x:si>
   <x:si>
@@ -444,6 +492,9 @@
     <x:t>3.24</x:t>
   </x:si>
   <x:si>
+    <x:t>P38995-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.25</x:t>
   </x:si>
   <x:si>
@@ -456,6 +507,9 @@
     <x:t>3.26</x:t>
   </x:si>
   <x:si>
+    <x:t>BD505A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.27</x:t>
   </x:si>
   <x:si>
@@ -477,6 +531,9 @@
     <x:t>3.29</x:t>
   </x:si>
   <x:si>
+    <x:t>P51911-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.30</x:t>
   </x:si>
   <x:si>
@@ -489,6 +546,9 @@
     <x:t>3.31</x:t>
   </x:si>
   <x:si>
+    <x:t>P52416-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.32</x:t>
   </x:si>
   <x:si>
@@ -510,6 +570,9 @@
     <x:t>3.34</x:t>
   </x:si>
   <x:si>
+    <x:t>P48183-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.35</x:t>
   </x:si>
   <x:si>
@@ -522,6 +585,9 @@
     <x:t>3.36</x:t>
   </x:si>
   <x:si>
+    <x:t>P48905-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.37</x:t>
   </x:si>
   <x:si>
@@ -534,6 +600,9 @@
     <x:t>3.38</x:t>
   </x:si>
   <x:si>
+    <x:t>P48920-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.39</x:t>
   </x:si>
   <x:si>
@@ -544,6 +613,9 @@
   </x:si>
   <x:si>
     <x:t>3.40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P52341-B21#0D1</x:t>
   </x:si>
   <x:si>
     <x:t>3.41</x:t>
@@ -1038,26 +1110,20 @@
       <x:c r="I3" s="0">
         <x:v>26632.75</x:v>
       </x:c>
-      <x:c r="R3" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W3" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" spans="1:27">
       <x:c r="A4" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
+      <x:c r="E4" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
       <x:c r="F4" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1066,23 +1132,20 @@
       </x:c>
       <x:c r="I4" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W4" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:27">
       <x:c r="A5" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
+      <x:c r="E5" s="0" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="F5" s="0">
         <x:v>2</x:v>
@@ -1093,23 +1156,20 @@
       <x:c r="I5" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W5" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="6" spans="1:27">
       <x:c r="A6" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
+      <x:c r="E6" s="0" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
       <x:c r="F6" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1118,23 +1178,20 @@
       </x:c>
       <x:c r="I6" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W6" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:27">
       <x:c r="A7" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
+      <x:c r="E7" s="0" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="F7" s="0">
         <x:v>2</x:v>
@@ -1145,23 +1202,20 @@
       <x:c r="I7" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W7" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" spans="1:27">
       <x:c r="A8" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
+      <x:c r="E8" s="0" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
       <x:c r="F8" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1170,24 +1224,21 @@
       </x:c>
       <x:c r="I8" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W8" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:27">
       <x:c r="A9" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
+      <x:c r="E9" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="F9" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1196,24 +1247,21 @@
       </x:c>
       <x:c r="I9" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W9" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:27">
       <x:c r="A10" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
+      <x:c r="E10" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
       <x:c r="F10" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1222,20 +1270,17 @@
       </x:c>
       <x:c r="I10" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W10" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:27">
       <x:c r="A11" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
         <x:v>54</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>52</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
         <x:v>55</x:v>
@@ -1248,9 +1293,6 @@
       </x:c>
       <x:c r="I11" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W11" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:27">
@@ -1261,10 +1303,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F12" s="0">
         <x:v>1</x:v>
@@ -1274,23 +1316,20 @@
       </x:c>
       <x:c r="I12" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W12" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:27">
       <x:c r="A13" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F13" s="0">
         <x:v>1</x:v>
@@ -1301,25 +1340,19 @@
       <x:c r="I13" s="0">
         <x:v>58842.8</x:v>
       </x:c>
-      <x:c r="R13" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W13" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" spans="1:27">
       <x:c r="A14" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F14" s="0">
         <x:v>1</x:v>
@@ -1329,23 +1362,20 @@
       </x:c>
       <x:c r="I14" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W14" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:27">
       <x:c r="A15" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F15" s="0">
         <x:v>1</x:v>
@@ -1355,23 +1385,20 @@
       </x:c>
       <x:c r="I15" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W15" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:27">
       <x:c r="A16" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F16" s="0">
         <x:v>1</x:v>
@@ -1381,23 +1408,20 @@
       </x:c>
       <x:c r="I16" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W16" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:27">
       <x:c r="A17" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F17" s="0">
         <x:v>1</x:v>
@@ -1407,23 +1431,20 @@
       </x:c>
       <x:c r="I17" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W17" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:27">
       <x:c r="A18" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F18" s="0">
         <x:v>1</x:v>
@@ -1433,23 +1454,20 @@
       </x:c>
       <x:c r="I18" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W18" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:27">
       <x:c r="A19" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F19" s="0">
         <x:v>1</x:v>
@@ -1459,23 +1477,20 @@
       </x:c>
       <x:c r="I19" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W19" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:27">
       <x:c r="A20" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F20" s="0">
         <x:v>1</x:v>
@@ -1485,23 +1500,20 @@
       </x:c>
       <x:c r="I20" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W20" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:27">
       <x:c r="A21" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F21" s="0">
         <x:v>1</x:v>
@@ -1511,23 +1523,20 @@
       </x:c>
       <x:c r="I21" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W21" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:27">
       <x:c r="A22" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="F22" s="0">
         <x:v>1</x:v>
@@ -1537,23 +1546,20 @@
       </x:c>
       <x:c r="I22" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W22" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:27">
       <x:c r="A23" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="F23" s="0">
         <x:v>1</x:v>
@@ -1563,23 +1569,20 @@
       </x:c>
       <x:c r="I23" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W23" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:27">
       <x:c r="A24" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="F24" s="0">
         <x:v>20</x:v>
@@ -1590,22 +1593,19 @@
       <x:c r="I24" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W24" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="25" spans="1:27">
       <x:c r="A25" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F25" s="0">
         <x:v>1</x:v>
@@ -1616,25 +1616,19 @@
       <x:c r="I25" s="0">
         <x:v>46237.81</x:v>
       </x:c>
-      <x:c r="R25" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W25" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" spans="1:27">
       <x:c r="A26" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F26" s="0">
         <x:v>1</x:v>
@@ -1644,23 +1638,20 @@
       </x:c>
       <x:c r="I26" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W26" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:27">
       <x:c r="A27" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F27" s="0">
         <x:v>1</x:v>
@@ -1670,23 +1661,20 @@
       </x:c>
       <x:c r="I27" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W27" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:27">
       <x:c r="A28" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F28" s="0">
         <x:v>1</x:v>
@@ -1696,23 +1684,20 @@
       </x:c>
       <x:c r="I28" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W28" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:27">
       <x:c r="A29" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F29" s="0">
         <x:v>1</x:v>
@@ -1722,23 +1707,20 @@
       </x:c>
       <x:c r="I29" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W29" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:27">
       <x:c r="A30" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F30" s="0">
         <x:v>4</x:v>
@@ -1749,22 +1731,19 @@
       <x:c r="I30" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W30" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="31" spans="1:27">
       <x:c r="A31" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F31" s="0">
         <x:v>4</x:v>
@@ -1775,22 +1754,19 @@
       <x:c r="I31" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W31" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="32" spans="1:27">
       <x:c r="A32" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F32" s="0">
         <x:v>1</x:v>
@@ -1800,23 +1776,20 @@
       </x:c>
       <x:c r="I32" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W32" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:27">
       <x:c r="A33" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F33" s="0">
         <x:v>1</x:v>
@@ -1826,23 +1799,20 @@
       </x:c>
       <x:c r="I33" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W33" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:27">
       <x:c r="A34" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F34" s="0">
         <x:v>1</x:v>
@@ -1852,23 +1822,20 @@
       </x:c>
       <x:c r="I34" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W34" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:27">
       <x:c r="A35" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F35" s="0">
         <x:v>1</x:v>
@@ -1878,23 +1845,20 @@
       </x:c>
       <x:c r="I35" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W35" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:27">
       <x:c r="A36" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F36" s="0">
         <x:v>1</x:v>
@@ -1904,23 +1868,20 @@
       </x:c>
       <x:c r="I36" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W36" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:27">
       <x:c r="A37" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F37" s="0">
         <x:v>1</x:v>
@@ -1930,23 +1891,20 @@
       </x:c>
       <x:c r="I37" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W37" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:27">
       <x:c r="A38" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E38" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F38" s="0">
         <x:v>1</x:v>
@@ -1956,23 +1914,20 @@
       </x:c>
       <x:c r="I38" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W38" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:27">
       <x:c r="A39" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F39" s="0">
         <x:v>1</x:v>
@@ -1982,23 +1937,20 @@
       </x:c>
       <x:c r="I39" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W39" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:27">
       <x:c r="A40" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="E40" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="F40" s="0">
         <x:v>1</x:v>
@@ -2008,23 +1960,20 @@
       </x:c>
       <x:c r="I40" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W40" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:27">
       <x:c r="A41" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E41" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F41" s="0">
         <x:v>1</x:v>
@@ -2034,23 +1983,20 @@
       </x:c>
       <x:c r="I41" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W41" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:27">
       <x:c r="A42" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E42" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F42" s="0">
         <x:v>1</x:v>
@@ -2060,23 +2006,20 @@
       </x:c>
       <x:c r="I42" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W42" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:27">
       <x:c r="A43" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E43" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F43" s="0">
         <x:v>1</x:v>
@@ -2086,23 +2029,20 @@
       </x:c>
       <x:c r="I43" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W43" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:27">
       <x:c r="A44" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E44" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="F44" s="0">
         <x:v>1</x:v>
@@ -2112,23 +2052,20 @@
       </x:c>
       <x:c r="I44" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W44" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:27">
       <x:c r="A45" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E45" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F45" s="0">
         <x:v>1</x:v>
@@ -2138,23 +2075,20 @@
       </x:c>
       <x:c r="I45" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W45" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:27">
       <x:c r="A46" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E46" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="F46" s="0">
         <x:v>1</x:v>
@@ -2164,23 +2098,20 @@
       </x:c>
       <x:c r="I46" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W46" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:27">
       <x:c r="A47" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E47" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F47" s="0">
         <x:v>1</x:v>
@@ -2190,23 +2121,20 @@
       </x:c>
       <x:c r="I47" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W47" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:27">
       <x:c r="A48" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E48" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F48" s="0">
         <x:v>2</x:v>
@@ -2217,22 +2145,19 @@
       <x:c r="I48" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W48" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="49" spans="1:27">
       <x:c r="A49" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E49" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F49" s="0">
         <x:v>2</x:v>
@@ -2243,22 +2168,19 @@
       <x:c r="I49" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W49" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="50" spans="1:27">
       <x:c r="A50" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E50" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="F50" s="0">
         <x:v>1</x:v>
@@ -2268,23 +2190,20 @@
       </x:c>
       <x:c r="I50" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W50" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:27">
       <x:c r="A51" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="E51" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F51" s="0">
         <x:v>1</x:v>
@@ -2294,23 +2213,20 @@
       </x:c>
       <x:c r="I51" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W51" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:27">
       <x:c r="A52" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D52" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E52" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="F52" s="0">
         <x:v>1</x:v>
@@ -2320,23 +2236,20 @@
       </x:c>
       <x:c r="I52" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W52" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:27">
       <x:c r="A53" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D53" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="E53" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="F53" s="0">
         <x:v>1</x:v>
@@ -2346,23 +2259,20 @@
       </x:c>
       <x:c r="I53" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W53" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:27">
       <x:c r="A54" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="E54" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F54" s="0">
         <x:v>1</x:v>
@@ -2372,23 +2282,20 @@
       </x:c>
       <x:c r="I54" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W54" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:27">
       <x:c r="A55" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E55" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F55" s="0">
         <x:v>1</x:v>
@@ -2398,23 +2305,20 @@
       </x:c>
       <x:c r="I55" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W55" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:27">
       <x:c r="A56" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E56" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F56" s="0">
         <x:v>1</x:v>
@@ -2424,23 +2328,20 @@
       </x:c>
       <x:c r="I56" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W56" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:27">
       <x:c r="A57" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D57" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E57" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F57" s="0">
         <x:v>1</x:v>
@@ -2450,23 +2351,20 @@
       </x:c>
       <x:c r="I57" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W57" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:27">
       <x:c r="A58" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D58" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="E58" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="F58" s="0">
         <x:v>1</x:v>
@@ -2476,23 +2374,20 @@
       </x:c>
       <x:c r="I58" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W58" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:27">
       <x:c r="A59" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D59" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="E59" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F59" s="0">
         <x:v>1</x:v>
@@ -2502,23 +2397,20 @@
       </x:c>
       <x:c r="I59" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W59" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:27">
       <x:c r="A60" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D60" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="E60" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="F60" s="0">
         <x:v>1</x:v>
@@ -2528,23 +2420,20 @@
       </x:c>
       <x:c r="I60" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W60" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:27">
       <x:c r="A61" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D61" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="E61" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F61" s="0">
         <x:v>1</x:v>
@@ -2554,23 +2443,20 @@
       </x:c>
       <x:c r="I61" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W61" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:27">
       <x:c r="A62" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D62" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E62" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F62" s="0">
         <x:v>1</x:v>
@@ -2580,23 +2466,20 @@
       </x:c>
       <x:c r="I62" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W62" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:27">
       <x:c r="A63" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D63" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E63" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F63" s="0">
         <x:v>1</x:v>
@@ -2606,23 +2489,20 @@
       </x:c>
       <x:c r="I63" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W63" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:27">
       <x:c r="A64" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D64" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E64" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="F64" s="0">
         <x:v>1</x:v>
@@ -2632,23 +2512,20 @@
       </x:c>
       <x:c r="I64" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W64" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:27">
       <x:c r="A65" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B65" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D65" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="E65" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F65" s="0">
         <x:v>1</x:v>
@@ -2658,23 +2535,20 @@
       </x:c>
       <x:c r="I65" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W65" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:27">
       <x:c r="A66" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D66" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="E66" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="F66" s="0">
         <x:v>1</x:v>
@@ -2684,23 +2558,20 @@
       </x:c>
       <x:c r="I66" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W66" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:27">
       <x:c r="A67" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D67" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E67" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F67" s="0">
         <x:v>1</x:v>
@@ -2710,23 +2581,20 @@
       </x:c>
       <x:c r="I67" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W67" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:27">
       <x:c r="A68" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D68" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="E68" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="F68" s="0">
         <x:v>1</x:v>
@@ -2736,17 +2604,14 @@
       </x:c>
       <x:c r="I68" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W68" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:27">
       <x:c r="B69" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D69" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
fix: update HPE bid line item output (#7)
## Summary

- append `OptionCode` to `ComponentID` with a `#` separator for HPE `BundleDetails` Vendor Part Numbers
- stop populating HPE Min Order Qty and Comments, using `Quantity` as the sole quantity source
- update the HPE extraction spec, output mapping, parser tests, and four sanitised golden workbooks
- ignore the root `/inbox/` directory so local supplier documents and analysis material cannot be committed

## Output changes

- `BundleDetails` with an option code now emit values such as `P72297-B21#ABG`; rows without one retain the base `ComponentID`
- CRM column R (Comments) and column W (Min Order Qty) are blank for all HPE Bid lines
- Part Number and Bundle option-code behavior is unchanged

## Validation

- `dotnet test BidParser.sln --no-restore` — 968 passed
- `npm run build` — passed
- both recent HPE samples parse successfully with option suffixes applied and no Min Order Qty or Comments values
</commit_message>
<xml_diff>
--- a/samples/outputs/HPE_Deal_9500000001_v2_NoCalculation.xlsx
+++ b/samples/outputs/HPE_Deal_9500000001_v2_NoCalculation.xlsx
@@ -114,9 +114,6 @@
     <x:t>MSL 2024 2xTLO-9 SAS</x:t>
   </x:si>
   <x:si>
-    <x:t>Max Qty: 1</x:t>
-  </x:si>
-  <x:si>
     <x:t>1.01</x:t>
   </x:si>
   <x:si>
@@ -183,12 +180,18 @@
     <x:t>1.08</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4B2A3#QC1</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE MSL TapeAssure Adv Lic Support</x:t>
   </x:si>
   <x:si>
     <x:t>1.09</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4B2A3#80N</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE MSL2024 Library Support</x:t>
   </x:si>
   <x:si>
@@ -222,6 +225,9 @@
     <x:t>2.03</x:t>
   </x:si>
   <x:si>
+    <x:t>R7M24A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Factory Integrated</x:t>
   </x:si>
   <x:si>
@@ -237,6 +243,9 @@
     <x:t>2.05</x:t>
   </x:si>
   <x:si>
+    <x:t>BB983A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>FACTORY INTEGRATED</x:t>
   </x:si>
   <x:si>
@@ -261,6 +270,9 @@
     <x:t>2.08</x:t>
   </x:si>
   <x:si>
+    <x:t>HU4A6A3#YHL</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE StoreOnce 3660 80TB Base System Supp</x:t>
   </x:si>
   <x:si>
@@ -276,6 +288,9 @@
     <x:t>2.10</x:t>
   </x:si>
   <x:si>
+    <x:t>HA124A1#5VF</x:t>
+  </x:si>
+  <x:si>
     <x:t>HPE StoreOnce 36xx Stup SVC</x:t>
   </x:si>
   <x:si>
@@ -309,6 +324,9 @@
     <x:t>3.02</x:t>
   </x:si>
   <x:si>
+    <x:t>P52499-B21#UUF</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.03</x:t>
   </x:si>
   <x:si>
@@ -321,6 +339,9 @@
     <x:t>3.04</x:t>
   </x:si>
   <x:si>
+    <x:t>P67079-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>Factory integrated</x:t>
   </x:si>
   <x:si>
@@ -336,6 +357,9 @@
     <x:t>3.06</x:t>
   </x:si>
   <x:si>
+    <x:t>P64706-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.07</x:t>
   </x:si>
   <x:si>
@@ -348,6 +372,9 @@
     <x:t>3.08</x:t>
   </x:si>
   <x:si>
+    <x:t>P48895-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.09</x:t>
   </x:si>
   <x:si>
@@ -360,6 +387,9 @@
     <x:t>3.10</x:t>
   </x:si>
   <x:si>
+    <x:t>804398-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.11</x:t>
   </x:si>
   <x:si>
@@ -372,6 +402,9 @@
     <x:t>3.12</x:t>
   </x:si>
   <x:si>
+    <x:t>P26259-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.13</x:t>
   </x:si>
   <x:si>
@@ -384,6 +417,9 @@
     <x:t>3.14</x:t>
   </x:si>
   <x:si>
+    <x:t>P01366-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.15</x:t>
   </x:si>
   <x:si>
@@ -396,6 +432,9 @@
     <x:t>3.16</x:t>
   </x:si>
   <x:si>
+    <x:t>P48918-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.17</x:t>
   </x:si>
   <x:si>
@@ -408,6 +447,9 @@
     <x:t>3.18</x:t>
   </x:si>
   <x:si>
+    <x:t>P58335-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.19</x:t>
   </x:si>
   <x:si>
@@ -420,6 +462,9 @@
     <x:t>3.20</x:t>
   </x:si>
   <x:si>
+    <x:t>P51181-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.21</x:t>
   </x:si>
   <x:si>
@@ -432,6 +477,9 @@
     <x:t>3.22</x:t>
   </x:si>
   <x:si>
+    <x:t>P48908-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.23</x:t>
   </x:si>
   <x:si>
@@ -444,6 +492,9 @@
     <x:t>3.24</x:t>
   </x:si>
   <x:si>
+    <x:t>P38995-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.25</x:t>
   </x:si>
   <x:si>
@@ -456,6 +507,9 @@
     <x:t>3.26</x:t>
   </x:si>
   <x:si>
+    <x:t>BD505A#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.27</x:t>
   </x:si>
   <x:si>
@@ -477,6 +531,9 @@
     <x:t>3.29</x:t>
   </x:si>
   <x:si>
+    <x:t>P51911-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.30</x:t>
   </x:si>
   <x:si>
@@ -489,6 +546,9 @@
     <x:t>3.31</x:t>
   </x:si>
   <x:si>
+    <x:t>P52416-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.32</x:t>
   </x:si>
   <x:si>
@@ -510,6 +570,9 @@
     <x:t>3.34</x:t>
   </x:si>
   <x:si>
+    <x:t>P48183-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.35</x:t>
   </x:si>
   <x:si>
@@ -522,6 +585,9 @@
     <x:t>3.36</x:t>
   </x:si>
   <x:si>
+    <x:t>P48905-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.37</x:t>
   </x:si>
   <x:si>
@@ -534,6 +600,9 @@
     <x:t>3.38</x:t>
   </x:si>
   <x:si>
+    <x:t>P48920-B21#0D1</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.39</x:t>
   </x:si>
   <x:si>
@@ -544,6 +613,9 @@
   </x:si>
   <x:si>
     <x:t>3.40</x:t>
+  </x:si>
+  <x:si>
+    <x:t>P52341-B21#0D1</x:t>
   </x:si>
   <x:si>
     <x:t>3.41</x:t>
@@ -1038,26 +1110,20 @@
       <x:c r="I3" s="0">
         <x:v>26632.75</x:v>
       </x:c>
-      <x:c r="R3" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W3" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" spans="1:27">
       <x:c r="A4" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
+      <x:c r="E4" s="0" t="s">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
       <x:c r="F4" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1066,23 +1132,20 @@
       </x:c>
       <x:c r="I4" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W4" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:27">
       <x:c r="A5" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
+      <x:c r="E5" s="0" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="F5" s="0">
         <x:v>2</x:v>
@@ -1093,23 +1156,20 @@
       <x:c r="I5" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W5" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="6" spans="1:27">
       <x:c r="A6" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
+      <x:c r="E6" s="0" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>41</x:v>
-      </x:c>
       <x:c r="F6" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1118,23 +1178,20 @@
       </x:c>
       <x:c r="I6" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W6" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:27">
       <x:c r="A7" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
+      <x:c r="E7" s="0" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>44</x:v>
       </x:c>
       <x:c r="F7" s="0">
         <x:v>2</x:v>
@@ -1145,23 +1202,20 @@
       <x:c r="I7" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W7" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" spans="1:27">
       <x:c r="A8" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
+      <x:c r="E8" s="0" t="s">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
       <x:c r="F8" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1170,24 +1224,21 @@
       </x:c>
       <x:c r="I8" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W8" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:27">
       <x:c r="A9" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
+      <x:c r="E9" s="0" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>50</x:v>
-      </x:c>
       <x:c r="F9" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1196,24 +1247,21 @@
       </x:c>
       <x:c r="I9" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W9" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:27">
       <x:c r="A10" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
+      <x:c r="E10" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
       <x:c r="F10" s="0">
         <x:v>1</x:v>
       </x:c>
@@ -1222,20 +1270,17 @@
       </x:c>
       <x:c r="I10" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W10" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:27">
       <x:c r="A11" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
         <x:v>54</x:v>
-      </x:c>
-      <x:c r="B11" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>52</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
         <x:v>55</x:v>
@@ -1248,9 +1293,6 @@
       </x:c>
       <x:c r="I11" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W11" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:27">
@@ -1261,10 +1303,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F12" s="0">
         <x:v>1</x:v>
@@ -1274,23 +1316,20 @@
       </x:c>
       <x:c r="I12" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W12" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:27">
       <x:c r="A13" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="F13" s="0">
         <x:v>1</x:v>
@@ -1301,25 +1340,19 @@
       <x:c r="I13" s="0">
         <x:v>58842.8</x:v>
       </x:c>
-      <x:c r="R13" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W13" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" spans="1:27">
       <x:c r="A14" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F14" s="0">
         <x:v>1</x:v>
@@ -1329,23 +1362,20 @@
       </x:c>
       <x:c r="I14" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W14" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:27">
       <x:c r="A15" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="F15" s="0">
         <x:v>1</x:v>
@@ -1355,23 +1385,20 @@
       </x:c>
       <x:c r="I15" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W15" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:27">
       <x:c r="A16" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F16" s="0">
         <x:v>1</x:v>
@@ -1381,23 +1408,20 @@
       </x:c>
       <x:c r="I16" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W16" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:27">
       <x:c r="A17" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="F17" s="0">
         <x:v>1</x:v>
@@ -1407,23 +1431,20 @@
       </x:c>
       <x:c r="I17" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W17" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:27">
       <x:c r="A18" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F18" s="0">
         <x:v>1</x:v>
@@ -1433,23 +1454,20 @@
       </x:c>
       <x:c r="I18" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W18" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:27">
       <x:c r="A19" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F19" s="0">
         <x:v>1</x:v>
@@ -1459,23 +1477,20 @@
       </x:c>
       <x:c r="I19" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W19" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:27">
       <x:c r="A20" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F20" s="0">
         <x:v>1</x:v>
@@ -1485,23 +1500,20 @@
       </x:c>
       <x:c r="I20" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W20" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:27">
       <x:c r="A21" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F21" s="0">
         <x:v>1</x:v>
@@ -1511,23 +1523,20 @@
       </x:c>
       <x:c r="I21" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W21" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:27">
       <x:c r="A22" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="F22" s="0">
         <x:v>1</x:v>
@@ -1537,23 +1546,20 @@
       </x:c>
       <x:c r="I22" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W22" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:27">
       <x:c r="A23" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="F23" s="0">
         <x:v>1</x:v>
@@ -1563,23 +1569,20 @@
       </x:c>
       <x:c r="I23" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W23" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:27">
       <x:c r="A24" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="F24" s="0">
         <x:v>20</x:v>
@@ -1590,22 +1593,19 @@
       <x:c r="I24" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W24" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="25" spans="1:27">
       <x:c r="A25" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F25" s="0">
         <x:v>1</x:v>
@@ -1616,25 +1616,19 @@
       <x:c r="I25" s="0">
         <x:v>46237.81</x:v>
       </x:c>
-      <x:c r="R25" s="0" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="W25" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="26" spans="1:27">
       <x:c r="A26" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F26" s="0">
         <x:v>1</x:v>
@@ -1644,23 +1638,20 @@
       </x:c>
       <x:c r="I26" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W26" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:27">
       <x:c r="A27" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F27" s="0">
         <x:v>1</x:v>
@@ -1670,23 +1661,20 @@
       </x:c>
       <x:c r="I27" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W27" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:27">
       <x:c r="A28" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F28" s="0">
         <x:v>1</x:v>
@@ -1696,23 +1684,20 @@
       </x:c>
       <x:c r="I28" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W28" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:27">
       <x:c r="A29" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F29" s="0">
         <x:v>1</x:v>
@@ -1722,23 +1707,20 @@
       </x:c>
       <x:c r="I29" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W29" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:27">
       <x:c r="A30" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F30" s="0">
         <x:v>4</x:v>
@@ -1749,22 +1731,19 @@
       <x:c r="I30" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W30" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="31" spans="1:27">
       <x:c r="A31" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F31" s="0">
         <x:v>4</x:v>
@@ -1775,22 +1754,19 @@
       <x:c r="I31" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W31" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="32" spans="1:27">
       <x:c r="A32" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="F32" s="0">
         <x:v>1</x:v>
@@ -1800,23 +1776,20 @@
       </x:c>
       <x:c r="I32" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W32" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:27">
       <x:c r="A33" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F33" s="0">
         <x:v>1</x:v>
@@ -1826,23 +1799,20 @@
       </x:c>
       <x:c r="I33" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W33" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:27">
       <x:c r="A34" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="F34" s="0">
         <x:v>1</x:v>
@@ -1852,23 +1822,20 @@
       </x:c>
       <x:c r="I34" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W34" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:27">
       <x:c r="A35" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F35" s="0">
         <x:v>1</x:v>
@@ -1878,23 +1845,20 @@
       </x:c>
       <x:c r="I35" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W35" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:27">
       <x:c r="A36" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F36" s="0">
         <x:v>1</x:v>
@@ -1904,23 +1868,20 @@
       </x:c>
       <x:c r="I36" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W36" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:27">
       <x:c r="A37" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F37" s="0">
         <x:v>1</x:v>
@@ -1930,23 +1891,20 @@
       </x:c>
       <x:c r="I37" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W37" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:27">
       <x:c r="A38" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="E38" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="F38" s="0">
         <x:v>1</x:v>
@@ -1956,23 +1914,20 @@
       </x:c>
       <x:c r="I38" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W38" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:27">
       <x:c r="A39" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F39" s="0">
         <x:v>1</x:v>
@@ -1982,23 +1937,20 @@
       </x:c>
       <x:c r="I39" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W39" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:27">
       <x:c r="A40" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="E40" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="F40" s="0">
         <x:v>1</x:v>
@@ -2008,23 +1960,20 @@
       </x:c>
       <x:c r="I40" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W40" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:27">
       <x:c r="A41" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="E41" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F41" s="0">
         <x:v>1</x:v>
@@ -2034,23 +1983,20 @@
       </x:c>
       <x:c r="I41" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W41" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:27">
       <x:c r="A42" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E42" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F42" s="0">
         <x:v>1</x:v>
@@ -2060,23 +2006,20 @@
       </x:c>
       <x:c r="I42" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W42" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:27">
       <x:c r="A43" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E43" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F43" s="0">
         <x:v>1</x:v>
@@ -2086,23 +2029,20 @@
       </x:c>
       <x:c r="I43" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W43" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:27">
       <x:c r="A44" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E44" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="F44" s="0">
         <x:v>1</x:v>
@@ -2112,23 +2052,20 @@
       </x:c>
       <x:c r="I44" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W44" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:27">
       <x:c r="A45" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="E45" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F45" s="0">
         <x:v>1</x:v>
@@ -2138,23 +2075,20 @@
       </x:c>
       <x:c r="I45" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W45" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:27">
       <x:c r="A46" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E46" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="F46" s="0">
         <x:v>1</x:v>
@@ -2164,23 +2098,20 @@
       </x:c>
       <x:c r="I46" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W46" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:27">
       <x:c r="A47" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E47" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F47" s="0">
         <x:v>1</x:v>
@@ -2190,23 +2121,20 @@
       </x:c>
       <x:c r="I47" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W47" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:27">
       <x:c r="A48" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E48" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F48" s="0">
         <x:v>2</x:v>
@@ -2217,22 +2145,19 @@
       <x:c r="I48" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W48" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="49" spans="1:27">
       <x:c r="A49" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E49" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F49" s="0">
         <x:v>2</x:v>
@@ -2243,22 +2168,19 @@
       <x:c r="I49" s="0">
         <x:v>0.0001</x:v>
       </x:c>
-      <x:c r="W49" s="0">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="50" spans="1:27">
       <x:c r="A50" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E50" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="F50" s="0">
         <x:v>1</x:v>
@@ -2268,23 +2190,20 @@
       </x:c>
       <x:c r="I50" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W50" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:27">
       <x:c r="A51" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="E51" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F51" s="0">
         <x:v>1</x:v>
@@ -2294,23 +2213,20 @@
       </x:c>
       <x:c r="I51" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W51" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:27">
       <x:c r="A52" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D52" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E52" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="F52" s="0">
         <x:v>1</x:v>
@@ -2320,23 +2236,20 @@
       </x:c>
       <x:c r="I52" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W52" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:27">
       <x:c r="A53" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D53" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="E53" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="F53" s="0">
         <x:v>1</x:v>
@@ -2346,23 +2259,20 @@
       </x:c>
       <x:c r="I53" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W53" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:27">
       <x:c r="A54" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="E54" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F54" s="0">
         <x:v>1</x:v>
@@ -2372,23 +2282,20 @@
       </x:c>
       <x:c r="I54" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W54" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:27">
       <x:c r="A55" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E55" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F55" s="0">
         <x:v>1</x:v>
@@ -2398,23 +2305,20 @@
       </x:c>
       <x:c r="I55" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W55" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:27">
       <x:c r="A56" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E56" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F56" s="0">
         <x:v>1</x:v>
@@ -2424,23 +2328,20 @@
       </x:c>
       <x:c r="I56" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W56" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:27">
       <x:c r="A57" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D57" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E57" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F57" s="0">
         <x:v>1</x:v>
@@ -2450,23 +2351,20 @@
       </x:c>
       <x:c r="I57" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W57" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="58" spans="1:27">
       <x:c r="A58" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D58" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="E58" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="F58" s="0">
         <x:v>1</x:v>
@@ -2476,23 +2374,20 @@
       </x:c>
       <x:c r="I58" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W58" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:27">
       <x:c r="A59" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D59" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="E59" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F59" s="0">
         <x:v>1</x:v>
@@ -2502,23 +2397,20 @@
       </x:c>
       <x:c r="I59" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W59" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:27">
       <x:c r="A60" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D60" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="E60" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="F60" s="0">
         <x:v>1</x:v>
@@ -2528,23 +2420,20 @@
       </x:c>
       <x:c r="I60" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W60" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:27">
       <x:c r="A61" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D61" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="E61" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F61" s="0">
         <x:v>1</x:v>
@@ -2554,23 +2443,20 @@
       </x:c>
       <x:c r="I61" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W61" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:27">
       <x:c r="A62" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D62" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E62" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F62" s="0">
         <x:v>1</x:v>
@@ -2580,23 +2466,20 @@
       </x:c>
       <x:c r="I62" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W62" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:27">
       <x:c r="A63" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D63" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E63" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F63" s="0">
         <x:v>1</x:v>
@@ -2606,23 +2489,20 @@
       </x:c>
       <x:c r="I63" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W63" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="64" spans="1:27">
       <x:c r="A64" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D64" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="E64" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="F64" s="0">
         <x:v>1</x:v>
@@ -2632,23 +2512,20 @@
       </x:c>
       <x:c r="I64" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W64" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="65" spans="1:27">
       <x:c r="A65" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="B65" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D65" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="E65" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F65" s="0">
         <x:v>1</x:v>
@@ -2658,23 +2535,20 @@
       </x:c>
       <x:c r="I65" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W65" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:27">
       <x:c r="A66" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D66" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="E66" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="F66" s="0">
         <x:v>1</x:v>
@@ -2684,23 +2558,20 @@
       </x:c>
       <x:c r="I66" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W66" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:27">
       <x:c r="A67" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D67" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="E67" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="F67" s="0">
         <x:v>1</x:v>
@@ -2710,23 +2581,20 @@
       </x:c>
       <x:c r="I67" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W67" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:27">
       <x:c r="A68" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D68" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="E68" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="F68" s="0">
         <x:v>1</x:v>
@@ -2736,17 +2604,14 @@
       </x:c>
       <x:c r="I68" s="0">
         <x:v>0.0001</x:v>
-      </x:c>
-      <x:c r="W68" s="0">
-        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:27">
       <x:c r="B69" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="D69" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>208</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>